<commit_message>
Add comment scraper and word cloud
</commit_message>
<xml_diff>
--- a/Data/7052019-09062024/Split_Data/with_account/Scraped_Results/N-VA_official.xlsx
+++ b/Data/7052019-09062024/Split_Data/with_account/Scraped_Results/N-VA_official.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,11 @@
           <t>hearts_count</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>transcription</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -481,10 +486,8 @@
           <t>yoleenvancamp</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>6829404014577274118</t>
-        </is>
+      <c r="B2" t="n">
+        <v>6.829404014577274e+18</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -515,6 +518,11 @@
       <c r="I2" t="n">
         <v>8</v>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>TRANSCRIPTION_FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -522,10 +530,8 @@
           <t>yoleenvancamp</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>6814781386495479046</t>
-        </is>
+      <c r="B3" t="n">
+        <v>6.814781386495479e+18</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -556,6 +562,11 @@
       <c r="I3" t="n">
         <v>14</v>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>TRANSCRIPTION_FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -563,10 +574,8 @@
           <t>yoleenvancamp</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>6800836810290236677</t>
-        </is>
+      <c r="B4" t="n">
+        <v>6.800836810290236e+18</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -597,6 +606,11 @@
       <c r="I4" t="n">
         <v>33</v>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>TRANSCRIPTION_FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -604,10 +618,8 @@
           <t>yoleenvancamp</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>6797406103211642118</t>
-        </is>
+      <c r="B5" t="n">
+        <v>6.797406103211642e+18</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -638,6 +650,11 @@
       <c r="I5" t="n">
         <v>123</v>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>You spin me right round baby Right Round like you like a baby Right Round Round Round</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -645,10 +662,8 @@
           <t>yoleenvancamp</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>6795993072367947013</t>
-        </is>
+      <c r="B6" t="n">
+        <v>6.795993072367947e+18</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -679,661 +694,2470 @@
       <c r="I6" t="n">
         <v>331</v>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>TRANSCRIPTION_FAILED</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>annickderidder.official</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>7205637927794134277</t>
-        </is>
+          <t>yoleenvancamp</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6.795673404314783e+18</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@annickderidder.official/video/7205637927794134277</t>
+          <t>https://www.tiktok.com/@yoleenvancamp/video/6795673404314782982</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1677693320</v>
+        <v>1582241023</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2023-03-01 09:55:20</t>
+          <t>2020-02-20 15:23:43</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Geen wandelende takken, maar wel schuivende bomen! Voor meer info over deze spectaculaire Antwerpse primeur in het #zuidpark, kijk VTM NIEUWS! #vergroening 🌳 ☀️</t>
+          <t>Tadaaa! #Pepper #foryourpage #dogsoftiktok #animallovers #mua #chihuahua gemaakt door academie Herentals ❤️</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>annickderidder.official</t>
+          <t>yoleenvancamp</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>33789</v>
+        <v>1722</v>
       </c>
       <c r="I7" t="n">
-        <v>587</v>
+        <v>104</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>TRANSCRIPTION_FAILED</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>annickderidder.official</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>7058532304406252806</t>
-        </is>
+          <t>yoleenvancamp</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>6.794526672944188e+18</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@annickderidder.official/video/7058532304406252806</t>
+          <t>https://www.tiktok.com/@yoleenvancamp/video/6794526672944188677</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1643442622</v>
+        <v>1581974022</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2022-01-28 23:50:22</t>
+          <t>2020-02-17 13:13:42</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>De Antwerpse haven blijft de grootste ter wereld hebben. Sorry, not sorry! ⚓?  (beelden VRT)  #antwerpen #antwerp #fyp #fy #portofantwerp #nederland #vlaanderen #haven #jobs #nieuws #tv</t>
+          <t>Net nu hij passé is onder de knie :-D #handchallenge #stipit #movetegenpesten</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>annickderidder.official</t>
+          <t>yoleenvancamp</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>54077</v>
+        <v>893</v>
       </c>
       <c r="I8" t="n">
-        <v>1711</v>
+        <v>22</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>TRANSCRIPTION_FAILED</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>bjanseeuw</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>7236030637944212763</t>
-        </is>
+          <t>yoleenvancamp</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>6.794055618027113e+18</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bjanseeuw/video/7236030637944212763</t>
+          <t>https://www.tiktok.com/@yoleenvancamp/video/6794055618027113733</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1684769689</v>
+        <v>1581864344</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2023-05-22 08:34:49</t>
+          <t>2020-02-16 06:45:44</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>𝗠𝗮𝗸𝗲-𝗼𝘃𝗲𝗿 𝗠𝗼𝗻𝗱𝗮𝘆 🤩 Opnieuw een stapje dichter bij een volledig vernieuwde handelskern, want ook de Hertstraat is afgewerkt! ✅</t>
+          <t>#duet met @luna.c.lunatic #elektrische #auto we zijn al met 2 😁 #duo</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>bjanseeuw</t>
+          <t>yoleenvancamp</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1044</v>
+        <v>27477</v>
       </c>
       <c r="I9" t="n">
-        <v>28</v>
+        <v>2939</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Jolene Jolene Jolene Jolene I love you Please Don't Take My Man</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>bjanseeuw</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>7227106970904349979</t>
-        </is>
+          <t>yoleenvancamp</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>6.794013163776986e+18</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bjanseeuw/video/7227106970904349979</t>
+          <t>https://www.tiktok.com/@yoleenvancamp/video/6794013163776986373</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1682691979</v>
+        <v>1581854460</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2023-04-28 07:26:19</t>
+          <t>2020-02-16 04:01:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Samen met heel wat helpende handen stak ik deze middag de handen uit de mouwen op de opruimactie in de wijk Nieuw Stene. 🚮 Even een shout-out naar onze medewerkers van de dienst Openbaar Domein die zich elke dag keihard inzetten om onze straten en pleinen proper te houden! 👏 Respect voor hun werk! 🙏</t>
+          <t>Sssht... onze Pepper helpt stiekem mee op benefiet spaghetti voor dierenasiel Unco-Jerry 😌 #chihuahua #nomnom #verstopt</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>bjanseeuw</t>
+          <t>yoleenvancamp</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>339</v>
+        <v>683</v>
       </c>
       <c r="I10" t="n">
-        <v>14</v>
+        <v>32</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>TRANSCRIPTION_FAILED</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>bjanseeuw</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>7224532772059204891</t>
-        </is>
+          <t>yoleenvancamp</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>6.793402371721514e+18</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bjanseeuw/video/7224532772059204891</t>
+          <t>https://www.tiktok.com/@yoleenvancamp/video/6793402371721514246</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1682092624</v>
+        <v>1581712248</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2023-04-21 08:57:04</t>
+          <t>2020-02-14 12:30:48</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>We duiken het weekend in met leuk nieuws! 🤩 Onze Christinastraat ligt er weer fantastisch bij! ✅ Ga jij dit weekend een kijkje nemen? 👀</t>
+          <t>#signlanguage #firstpost #jolene</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>bjanseeuw</t>
+          <t>yoleenvancamp</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1106</v>
+        <v>193</v>
       </c>
       <c r="I11" t="n">
-        <v>26</v>
+        <v>9</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Joling</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>bjanseeuw</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>7199537458885807366</t>
-        </is>
+          <t>annickderidder.official</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>7.205637927794134e+18</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bjanseeuw/video/7199537458885807366</t>
+          <t>https://www.tiktok.com/@annickderidder.official/video/7205637927794134277</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1676272955</v>
+        <v>1677693320</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2023-02-12 23:22:35</t>
+          <t>2023-03-01 09:55:20</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>𝗠𝗮𝗸𝗲-𝗼𝘃𝗲𝗿 𝗠𝗼𝗻𝗱𝗮𝘆 🤩 Had je het al gemerkt? Onze Amandine straalt opnieuw, en hoe! Fantastisch dat we dankzij de renovatie van de romp van het schip weer kunnen genieten van dit iconisch stukje Oostende!  En het goede nieuws is: ook de werken aan het museum, onderaan het schip, starten binnenkort. Je zal onze Amandine dus snel opnieuw kunnen bezoeken, iets om naar uit te kijken!</t>
+          <t>Geen wandelende takken, maar wel schuivende bomen! Voor meer info over deze spectaculaire Antwerpse primeur in het #zuidpark, kijk VTM NIEUWS! #vergroening 🌳 ☀️</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>bjanseeuw</t>
+          <t>annickderidder.official</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1067</v>
+        <v>33789</v>
       </c>
       <c r="I12" t="n">
-        <v>15</v>
+        <v>587</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>in Antwerpen worden een aantal bomen verplaatst voor de heraanleg van de Gedempte zuiderdokken de vroegere parking wordt nu een park van 7 hectare de bomen die er al stonden worden niet met wortelen al uitgegraven maar verschoven zo blijft de kluit beter beschermd en zou de boom langer mee gaan een beetje op af en ook Patrick bon verzorger Stijn de Tafelen is verhuisd coördinator van een jonge zomer Eik van 23 jaar wordt verplaatst en dat doen ze op een bijzondere manier we hebben eerst de kleuter rond gegraven dan hebben we kettingen er onder getrokken om uiteindelijk te onderzoeken en dan hebben we platen onder getrokken die platen hebben we verbonden aan elkaar zodat we één pakket hebben zodat we eigenlijk de kleuters de grote die we willen die nodig is voor een boom volledig kunnen verschuiven het plaatsen van de en de kettingen plus het verplaatsen van een boom duurt een volledige werkdag op deze manier beperk je wel de wortels schade en kan de boom nog jaren mee dus nu straks als je een op zijn definitieve plaats staat hadden we dan ook nog de groepen zijn groei plaats optimaliseren zodat hij voor de komende 50 jaar eindelijk eh voedingsstoffen genoeg heeft de bomen verhuis maakt del uit van de aanleg van het nieuwe zuidpark in Antwerpen beter bekend als de oude Gedempte zuiderdokken ooit de vaste St de sinksenfoor en de meest bekende gratis openlucht parking van de stad die wagens die zijn nu onder de grond gebracht en eh boven de grond maken werk van een park van marlies zeven hectare met de meer dan 30.000 nieuwe planten 497 bomen dus dat wordt hier een ja van fantastische plek voor iedereen die hier woont maar ook komt eh naar antwerpen-zuid komt komt wandelen komt bezoeken het park wordt in verschillende fases afgewerkt en moet volledig klaar zijn in de lente volgend jaar</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>bjanseeuw</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>7190685985129254149</t>
-        </is>
+          <t>annickderidder.official</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>7.058532304406253e+18</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bjanseeuw/video/7190685985129254149</t>
+          <t>https://www.tiktok.com/@annickderidder.official/video/7058532304406252806</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1674212056</v>
+        <v>1643442622</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2023-01-20 02:54:16</t>
+          <t>2022-01-28 23:50:22</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Deze zondag 22/01 nieuwjaarsreceptie van N-VA Oostende, met deze topper Theo Francken! 🙌  Iedereen is van harte welkom, inschrijven is niet nodig. 🤩 Tot dan? 😁</t>
+          <t>De Antwerpse haven blijft de grootste ter wereld hebben. Sorry, not sorry! ⚓?  (beelden VRT)  #antwerpen #antwerp #fyp #fy #portofantwerp #nederland #vlaanderen #haven #jobs #nieuws #tv</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>bjanseeuw</t>
+          <t>annickderidder.official</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1428</v>
+        <v>54089</v>
       </c>
       <c r="I13" t="n">
-        <v>27</v>
+        <v>1713</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Waar ligt de grootste Sluis van de wereld wel de topscorer die is er voor Kallo bij bijvullen de Antwerpse haven dus daar is de grootste Sluis van de wereld sinds 2016 en er zijn ook bonuspunten voor de naam Het is de kieldrechtsluis de grootste van de wereld Dat dachten wij toch want eh deze middag gehoord dat het volgende op het NOS journaal koning willem-alexander heeft de zeesluis IJmuiden officieel geopend Het is de grootste thuis ter wereld aan ander verkeer bij IJmuiden de binnendeur van zeesluis IJmuiden is open de deur is open van die sluis bij IJmuiden Dus we gaan er eens naar kijken de afmetingen 500 meter lang is ze ze is 70 meter breed en ook 18 meter diep houd die afmetingen goed vast zou ik zeggen want nu leggen we die Kieldrecht is er langs en die is eh Jawel ook 500 meter lang maar slechts 68 meter breed en ook minder diep Ze is 17,8 M qua dit Oké dat is dus minder breed om die nieuwe sluis in Nederland minder diep ook dat zou je toch denken maar eh nee nee niks van dat zegt de volgende man en hij kan het eigenlijk wel weten want het is een man die jarenlang Haven Ingenieur geweest is er is een verschil tussen referentie pijlen in Nederland en in België het Belgische pijl is gerefereerd naar de laagwaterstand de gemiddelde dagwaarde stand in Oostende het Nederlandse pijl is refereert naar de gemiddelde waterstand in op zee droogte van IJmuiden maar dat is gevolg dat er een niveauverschil is van ongeveer 2 meter 33 Met als gevolg Ja dat het ook het volume eh want bij de Solaris en verschil met eh de berekening geeft dan ongeveer 7% ja dat is ongeveer 7% in het voordeel van de kieldrechtsluis die Sluis blijft dus de grootste van de wereld en nu wil ik echt niks zeggen over de antwerpenaar hè maar Oh jawel daar zijn ze blij ja ik was heel verheugd om dat te horen eigenlijk hè Want het was was er een man van het Groenewoud al zong Ik wil de grootste heb ik wil altijd de grootste hebben dan ook heel blij als ze haven schepen dat ik de grootste heb kieldrechtsluis maar het is natuurlijk meer dan dat en eh ja dag en nacht werken en 150000 mensen eraan om ook de meest efficiënte performante en productieve haven te zijn en dat is uiteindelijk hotel Gooi Ja maar dat is toch vooral wat ik onthoud</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>koen.metsu.tiktok</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>7377664760298491169</t>
-        </is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7.236030637944212e+18</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7377664760298491169</t>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7236030637944212763</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1717746444</v>
+        <v>1684769689</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2024-06-07 00:47:24</t>
+          <t>2023-05-22 08:34:49</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>10 Jaar geleden heb ik voor het eerst mijn sprong in het parlement gewaagd en de rest is toekomst… 🪂</t>
+          <t>𝗠𝗮𝗸𝗲-𝗼𝘃𝗲𝗿 𝗠𝗼𝗻𝗱𝗮𝘆 🤩 Opnieuw een stapje dichter bij een volledig vernieuwde handelskern, want ook de Hertstraat is afgewerkt! ✅</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>koen.metsu.tiktok</t>
+          <t>bjanseeuw</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1944</v>
+        <v>1044</v>
       </c>
       <c r="I14" t="n">
-        <v>122</v>
+        <v>28</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>koen.metsu.tiktok</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>7376657454727286048</t>
-        </is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>7.22710697090435e+18</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7376657454727286048</t>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7227106970904349979</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1717511912</v>
+        <v>1682691979</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2024-06-04 07:38:32</t>
+          <t>2023-04-28 07:26:19</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Samen veilig METsU #7 Elisabet Haesevoets, dokter in de esthetische geneeskunde en de mol in 2019  #6 #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen</t>
+          <t>Samen met heel wat helpende handen stak ik deze middag de handen uit de mouwen op de opruimactie in de wijk Nieuw Stene. 🚮 Even een shout-out naar onze medewerkers van de dienst Openbaar Domein die zich elke dag keihard inzetten om onze straten en pleinen proper te houden! 👏 Respect voor hun werk! 🙏</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>koen.metsu.tiktok</t>
+          <t>bjanseeuw</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>11741</v>
+        <v>339</v>
       </c>
       <c r="I15" t="n">
-        <v>186</v>
+        <v>14</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>la sou</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>koen.metsu.tiktok</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>7374728766997777697</t>
-        </is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7.224532772059205e+18</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7374728766997777697</t>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7224532772059204891</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1717062853</v>
+        <v>1682092624</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2024-05-30 02:54:13</t>
+          <t>2023-04-21 08:57:04</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Samen veilig METsU #6 @kraftmeister Nick Kraft, Den Iejenigen Echten @djronnyretro bekend uit Big Brother</t>
+          <t>We duiken het weekend in met leuk nieuws! 🤩 Onze Christinastraat ligt er weer fantastisch bij! ✅ Ga jij dit weekend een kijkje nemen? 👀</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>koen.metsu.tiktok</t>
+          <t>bjanseeuw</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>11657</v>
+        <v>1106</v>
       </c>
       <c r="I16" t="n">
-        <v>118</v>
+        <v>26</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>koen.metsu.tiktok</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>7371399088887106848</t>
-        </is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>7.199537458885807e+18</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7371399088887106848</t>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7199537458885807366</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1716287605</v>
+        <v>1676272955</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2024-05-21 03:33:25</t>
+          <t>2023-02-12 23:22:35</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Samen veilig METsU #5 Jean-Marie Pfaff, Rode Duivel en legendarische doelman van Bayern München #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen #</t>
+          <t>𝗠𝗮𝗸𝗲-𝗼𝘃𝗲𝗿 𝗠𝗼𝗻𝗱𝗮𝘆 🤩 Had je het al gemerkt? Onze Amandine straalt opnieuw, en hoe! Fantastisch dat we dankzij de renovatie van de romp van het schip weer kunnen genieten van dit iconisch stukje Oostende!  En het goede nieuws is: ook de werken aan het museum, onderaan het schip, starten binnenkort. Je zal onze Amandine dus snel opnieuw kunnen bezoeken, iets om naar uit te kijken!</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>koen.metsu.tiktok</t>
+          <t>bjanseeuw</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>3437</v>
+        <v>1067</v>
       </c>
       <c r="I17" t="n">
-        <v>54</v>
+        <v>15</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>koen.metsu.tiktok</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>7369537323953917217</t>
-        </is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>7.190685985129254e+18</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7369537323953917217</t>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7190685985129254149</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1715854160</v>
+        <v>1674212056</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2024-05-16 03:09:20</t>
+          <t>2023-01-20 02:54:16</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Ik kom normaal zelden uit de lucht gevallen maar in aanloop naar 9 juni maak ik voor 1 keer een uitzondering… 🪂✈️ #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen</t>
+          <t>Deze zondag 22/01 nieuwjaarsreceptie van N-VA Oostende, met deze topper Theo Francken! 🙌  Iedereen is van harte welkom, inschrijven is niet nodig. 🤩 Tot dan? 😁</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>koen.metsu.tiktok</t>
+          <t>bjanseeuw</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>3316</v>
+        <v>1428</v>
       </c>
       <c r="I18" t="n">
-        <v>67</v>
+        <v>27</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>beste vrienden uit Oostende en omstreken ik mag jullie uitnodigen nu zondag in het clubhuis van de oostendse roeiclub langs de Prins Albertlaan vanaf 11 uur voor onze bijzonder boeiende nieuwjaarsreceptie want daar zal aanwezig zijn niemand minder dan deze topper dank beste mensen Zondag ben ik in Oostende samen Bjorn vele andere jullie een gelukkig nieuwjaar wensen maar vooral het hebben over het land waar gaan we naartoe Vlaanderen Waar gaat het naartoe twisten wat met die oorlog in Oekraïne Wat is de toekomst voor het westen België Vlaanderen en Oostende dag tot zondag</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>kathleen.depoorter</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>7348899495326829856</t>
-        </is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>7.175037729791561e+18</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kathleen.depoorter/video/7348899495326829856</t>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7175037729791560966</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1711049062</v>
+        <v>1670568660</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2024-03-21 12:24:22</t>
+          <t>2022-12-08 22:51:00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Preventie, vroege diagnose en nieuwe therapieën zijn essentieel in de strijd tegen #kanker. Als N-VA pleiten we voor een nieuw kankerplan met een gerichte aanpak en bijzondere aandacht voor prostaatkanker en longkanker.</t>
+          <t>Vanaf 1 januari 2023 worden de bewonerskaarten in Oostende gedigitaliseerd 🤩</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>kathleen.depoorter</t>
+          <t>bjanseeuw</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>390</v>
+        <v>455</v>
       </c>
       <c r="I19" t="n">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>vanaf 1 januari 2023 worden ook de bewoners kaarten in Oostende volledig gedigitaliseerd Dat betekent dat je vanaf nieuwjaar je papier bewoners kaart niet langer zichtbaar in je wagen moet leggen let wel tot nieuwjaar moet je dat nog altijd wel doen Wat moet je doen om die digitale bewoners kaart te krijgen als je bewoners kaart eind dit jaar afloopt dan moet je sowieso een nieuwe bonuskaart aanvragen Dat kan op deze website dat kan ook in het parkeren als je bewoners kaart nog geldig eind volgend jaar hoef je helemaal niks te doen die bewoners kaarten worden automatisch gedigitaliseerd natuurlijk moet je eind volgend jaar dan wel opnieuw een verlenging aanvragen</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>kathleen.depoorter</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>7340979348725304609</t>
-        </is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>7.172441934370278e+18</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kathleen.depoorter/video/7340979348725304609</t>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7172441934370278662</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1709204963</v>
+        <v>1669964281</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2024-02-29 03:09:23</t>
+          <t>2022-12-01 22:58:01</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Regelmatig krijg ik vragen over #Ozempic. Als apotheker en #parlementslid ben ik me bewust van het tekort, niet alleen van Ozempic-pennen, maar ook van andere #medicatie. Om dit probleem aan te pakken, heeft de #N-VA enkele jaren geleden een wetsvoorstel ingediend. Het voorstel is ondertussen goedgekeurd maar de uitvoering ervan door Minister Vandenbroucke laat nog op zich wachten. Ik volg het alvast op voor u!</t>
+          <t>Parkeren voor personen met een handicap blijft GRATIS in Oostende! 👌</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>kathleen.depoorter</t>
+          <t>bjanseeuw</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>93</v>
+        <v>687</v>
       </c>
       <c r="I20" t="n">
-        <v>7</v>
+        <v>21</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>personen een handicap kun je in Oostende onbeperkt parkeren op de openbare weg behalve opblazen voor zorgverstrekkers bewoners en Praxis Bovendien kunnen ze nog volledig gratis doen het enige wat ze moeten doen om het grafisch parkeren te behouden na nieuwjaar ik zeg eenmalig registreren in ons parkeerplaats of op deze website Je kan daar boven die niet heen maar twee nummerplaten registreren zo kan u blijven gaan en staan waar u maar wilt makkelijk toch</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>kathleen.depoorter</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>7338354886922390816</t>
-        </is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>7.172073007869857e+18</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kathleen.depoorter/video/7338354886922390816</t>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7172073007869857030</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1708593935</v>
+        <v>1669878381</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2024-02-22 01:25:35</t>
+          <t>2022-11-30 23:06:21</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1048 #jongeren tussen 18 en 24 jaar werden er in 2021 in gedwongen opnames geplaatst. Dat zijn er 35% meer dan in het jaar 2017. Deze stijging is het zoveelste signaal dat het niet goed gaat met het mentaal welzijn van onze jeugd. Er moet dringend meer ingezet worden op #preventie en sensibilisering, meer ambulante zorg en we hebben nood aan meer zorgverstrekkers gespecialiseerd in geestelijke #gezondheidszorg !</t>
+          <t>De jeton blijft! 🥳 #parkeren #inoostende #parkeerbeleid #30mingratis</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>kathleen.depoorter</t>
+          <t>bjanseeuw</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>912</v>
+        <v>2499</v>
       </c>
       <c r="I21" t="n">
-        <v>12</v>
+        <v>82</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2 jetons de Hello digitale versie dan is je nummerplaat eenmalig registreren in het parkeerloket of op deze website in één keer dat hebt gedaan dan kun je een gratis parkeren door je nummerplaat in te geven op de nieuwe parkeerautomaten makkelijk toch Oh ja mensen die bewoners kaart hebben moeten de eenmalige registratie van een nummerplaat niet eens doen Zij kunnen onmiddellijk op de nieuwe parkeerautomaten en gratis parkeren sessie van dus dat het door hun nummerplaat daar in te geven</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>7.159172831350377e+18</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7159172831350377733</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1666874822</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2022-10-27 05:47:02</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Met deze splinternieuwe automatische schuifdeuren aan beide ingangen van ons Conservatorium aan Zee halen we niet alleen de energiefactuur naar beneden, het gebouw wordt zo ook een stuk veiliger. 🎼</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>1213</v>
+      </c>
+      <c r="I22" t="n">
+        <v>36</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>7.15074214815184e+18</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7150742148151840006</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1664911902</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2022-10-04 12:31:42</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>De kerkhofmuur van Stene straalt opnieuw! ⛪️</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>933</v>
+      </c>
+      <c r="I23" t="n">
+        <v>18</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>et ouais ouais</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>7.145498407568788e+18</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7145498407568788742</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1663691000</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2022-09-20 09:23:20</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Of we in Oostende voor veel stadsvernieuwing zorgen? 😉 #oostende #stadoostende #stadsvernieuwing #lintjesknippen #kunnenwe #doenwe #loveoostende</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>1665</v>
+      </c>
+      <c r="I24" t="n">
+        <v>17</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>7.142924588681399e+18</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7142924588681399558</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1663091735</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2022-09-13 10:55:35</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Ontdek de locaties van de 7 nieuwe afvalstraten 📍#oostende #stadoostende #afvalstraat #stadsvernieuwing #tiktoktuesday</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>294</v>
+      </c>
+      <c r="I25" t="n">
+        <v>5</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>7.140329381846617e+18</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7140329381846617350</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1662487489</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2022-09-06 11:04:49</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Vastberaden om alle Oostendse schoolomgevingen veiliger te maken 💪 #oostende #stadoostende #veiligheid #veilige #school #omgeving #kunnenwe #doenwe #stadsvernieuwing</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>1888</v>
+      </c>
+      <c r="I26" t="n">
+        <v>28</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>7.137582091461545e+18</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7137582091461545222</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1661847839</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2022-08-30 01:23:59</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Come check this 🙌 #oostende #stadoostende #stadsvernieuwing #makeover #comecheckthis #afvalstraat #afval #tegenafval #netheid #nettestad #kunnenwe #tiktoktuesday</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>1722</v>
+      </c>
+      <c r="I27" t="n">
+        <v>23</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>kom check this</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>7.13508502980107e+18</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7135085029801069829</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1661266446</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2022-08-23 07:54:06</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Wist je dat we deze bestuursperiode al meer dan 20 km fietspad (her)aanlegden? 🤩 #oostende #stadoostende #stadsvernieuwing #fietsen #fietsstad #kunnenwe #doenwe #tiktoktuesday</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>10481</v>
+      </c>
+      <c r="I28" t="n">
+        <v>70</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>7.132354410574892e+18</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7132354410574892293</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1660630683</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2022-08-15 23:18:03</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>📍 Duinkerkseweg ➕2,3 km extra nieuw aangelegde fietspaden 🤩 #oostende #stadoostende #fietsen #fietspad #fietsstad #stadsvernieuwing #loveoostende #tiktoktuesday</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>1353</v>
+      </c>
+      <c r="I29" t="n">
+        <v>14</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>7.129882578080861e+18</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7129882578080861446</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1660055154</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2022-08-09 07:25:54</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Opnieuw een veilige oversteekplaats erbij ✅ #veiligheid #veiligheidboven #oversteekplaats #oostende #loveoostende #tiktoktuesday #stadsvernieuwing</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>146</v>
+      </c>
+      <c r="I30" t="n">
+        <v>4</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>7.127184023364881e+18</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7127184023364881669</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1659426852</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2022-08-02 00:54:12</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1 2 3 4 💥 #oostende #stadoostende #loveoostende #voetpad #vernieuwd #stadsvernieuwing #tiktoktuesday</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>3295</v>
+      </c>
+      <c r="I31" t="n">
+        <v>53</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>7.124595864277913e+18</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7124595864277912838</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1658824247</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2022-07-26 01:30:47</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Heraanleg stationsplein Oostende 🤩 #geslaagd #stationsplein #oostende #loveoostende #stadoostende #stadsvernieuwing #tiktoktuesday</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>826</v>
+      </c>
+      <c r="I32" t="n">
+        <v>18</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>7.122707472166505e+18</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7122707472166505734</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1658384573</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2022-07-20 23:22:53</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Out of office 😎 #holiday #vacation #vacaymode #fijnevakantie #outofoffice #oostende #loveoostende</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>517</v>
+      </c>
+      <c r="I33" t="n">
+        <v>12</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>7.12197033247433e+18</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7121970332474330373</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1658212942</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2022-07-18 23:42:22</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Hopla! 🤩 nog een vernieuwd fietspad, zo vlak als een biljart! 🎱 #oostende #stadoostende #loveoostende #fiets #fietsen #fietspad #fietsstad #tiktoktuesday</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>11372</v>
+      </c>
+      <c r="I34" t="n">
+        <v>153</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Sam Barry world to me the world is gonna</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>7.11935746736397e+18</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7119357467363970310</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1657604591</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2022-07-11 22:43:11</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Make-over van de atletiekpiste op de Schorre! 🤩 #kunnenwe #oostende #stadoostende #stadsvernieuwing #atletiek #atletiekpiste #ticktickboom #makeover</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>1502</v>
+      </c>
+      <c r="I35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>tu étais bon</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>7.116761760236948e+18</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7116761760236948741</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1657000230</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2022-07-04 22:50:30</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Een nieuw bloemenuurwerk, als ode aan onze Arno 💐 #oostende #stadoostende #bloemenuurwerk #ode #arno #vivre #jeveuxvivre</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>605</v>
+      </c>
+      <c r="I36" t="n">
+        <v>11</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>je veux vivre dans ce monde sans pilule où les riches et les pauvres n'existent plus</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>7.11417702293447e+18</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@bjanseeuw/video/7114177022934469894</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1656398421</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2022-06-27 23:40:21</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Van 6 naar 64 fietsstraten in Oostende! 💪 #oostende #stadoostende  #stadsvernieuwing #fietsstraten #bjornanseeuw #nva #schepen</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>bjanseeuw</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>6777</v>
+      </c>
+      <c r="I37" t="n">
+        <v>123</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Wat zijn jullie fantastisch</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>7.377664760298491e+18</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7377664760298491169</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1717746444</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2024-06-07 00:47:24</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>10 Jaar geleden heb ik voor het eerst mijn sprong in het parlement gewaagd en de rest is toekomst… 🪂</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>1944</v>
+      </c>
+      <c r="I38" t="n">
+        <v>122</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>10 jaar geleden werd ik de Sprong in het parlement spannend en soms met tegenwind maar omringd door de juiste mensen kunnen onze doelen bereiken mijn naam is Koen met Sue en sinds die dag mag ik mij inzetten voor het uw veiligheid als voorzitter van de politie en bij aan het wezen reservist in het leger en voorstellen we dat doen maatje commissie terreurbestrijding weet ik welke uitdagingen op ons afkomen met uw steun marco samen een einde aan die straffeloosheid want uw veiligheid moet terug bovenaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>7.376657454727286e+18</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7376657454727286048</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1717511912</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2024-06-04 07:38:32</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Samen veilig METsU #7 Elisabet Haesevoets, dokter in de esthetische geneeskunde en de mol in 2019  #6 #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>11741</v>
+      </c>
+      <c r="I39" t="n">
+        <v>186</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>als jij hier straks meer wat kan ik je echt rennen dat is anders weet je als je op controle gaat bij de oogarts en ik kijk die oogdruk naar is in dat opzicht heb ik wel als Ja het idealisme eigenlijk urgentie geen eens kunnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>7.374728766997777e+18</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7374728766997777697</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1717062853</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2024-05-30 02:54:13</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Samen veilig METsU #6 @kraftmeister Nick Kraft, Den Iejenigen Echten @djronnyretro bekend uit Big Brother</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>11657</v>
+      </c>
+      <c r="I40" t="n">
+        <v>118</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Heb jij iets bij kan jij regelen maar ik heb dat gij dan denk ik toch Ik heb dat nog nooit gedaan en toch komen die mensen naar mij</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>7.371399088887107e+18</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7371399088887106848</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1716287605</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2024-05-21 03:33:25</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Samen veilig METsU #5 Jean-Marie Pfaff, Rode Duivel en legendarische doelman van Bayern München #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen #</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>3437</v>
+      </c>
+      <c r="I41" t="n">
+        <v>54</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Carmen is daar slachtoffer geworden van een hele brutale homejacking Waar zijn die bek waarschijnlijk met museum hier in Beveren en ik ben naar huis gekomen en te onderweg kreeg ik telefoon van ons links en papa weet ik ook wel gemaakt en hij vertelde dat de mama overvallen was</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>7.369537323953917e+18</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7369537323953917217</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>1715854160</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2024-05-16 03:09:20</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Ik kom normaal zelden uit de lucht gevallen maar in aanloop naar 9 juni maak ik voor 1 keer een uitzondering… 🪂✈️ #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>3316</v>
+      </c>
+      <c r="I42" t="n">
+        <v>67</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>10 jaar geleden werd ik de Sprong in het parlement spannend en soms met tegenwind maar omringd door de juiste mensen kunnen onze doelen bereiken mijn naam is Koen met Sue en sinds die dag mag ik mij inzetten voor het uw veiligheid als voorzitter van de politie en bij aan het wezen reserves in het leger en voorstellen we dat doen maatje commissie terreurbestrijding weet ik welke uitdagingen op ons afkomen met uw steun marco samen een einde aan die straffeloosheid want uw veiligheid moet terug bovenaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>7.369150332414316e+18</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7369150332414315808</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>1715764028</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2024-05-15 02:07:08</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Samen veilig METsU #4 Willem Van Hoeck, LO-leerkracht bekend van Kamp Waes #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>9496</v>
+      </c>
+      <c r="I43" t="n">
+        <v>198</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Ik wou echt dat wij dezelfde middelen kregen als City Pirates om zo'n buurtsport te uit te breiden want dat was dat die doen met huiswerkbegeleiding mee opvang en zo dat is dat is natuurlijk nog nog drie gradaties ja ja ja ja ja ja die hebben echt een eh van uus opvang</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>7.368512293631528e+18</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7368512293631528225</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1715615468</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2024-05-13 08:51:08</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Wie is de man op plaats 6 voor de Kamer? Ontdek het hier. De muziek is een prachtige cover van Lean on Me door Jan Kerckhofs.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>1361</v>
+      </c>
+      <c r="I44" t="n">
+        <v>22</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DOWNLOAD_FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>7.366631902406626e+18</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7366631902406626593</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>1715177656</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2024-05-08 07:14:16</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Vraag van de dag: Hoe kijk je terug op een legislatuur oppositie? #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>1286</v>
+      </c>
+      <c r="I45" t="n">
+        <v>8</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Dat is niks voor mij ik vind eigenlijk heel weinig productief om in een oppositie te zitten natuurlijk wat we gedaan hebben is onze Job hè We hebben Vivaldi op een tekortkoming geweest en Helaas waren die wel Legio maar ik ben iemand die dat wilt wil besturen met de knoppen zitten beleid voeren verantwoordelijk zijn vanuit oppositie is het altijd heel gemakkelijk om om te roeptoeter en te zeggen het is niet goed en wij komen zelf met heel veel goede initiatieven maar dat politieke spel vandaag de dag is nog altijd wel het is komt het vanuit de Opel positie dan wordt het zo goed als zeker eh niet gestemd of niet goedgekeurd en eh dat soms frustrerend</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>7.365880513782959e+18</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7365880513782959393</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1715002710</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2024-05-06 06:38:30</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Samen veilig METsU #2 Glali Bnani, eigenaar van Glali Gym &amp; KickOff Sports #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>1442</v>
+      </c>
+      <c r="I46" t="n">
+        <v>49</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>hoe dat je verkeerd dat draait de jeugd is de toekomst hè En het is mijn mijn doel mijn tak om de jeugd veer Barden te maken sterker te maken en dat doe ik door middel van eh sport aan te bieden</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>7.364720884277333e+18</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7364720884277333280</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1714732716</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2024-05-03 03:38:36</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Throwback naar de aanloop van de verkiezingen in 2019, hou zeker mijn sociale media in de gaten voor de remake in 2024. In dit filmpje leer je me nog beter kennen. Wie is de man op plaats 6 voor de Kamer? Ontdek het hier. De muziek is een prachtige cover van High Hopes door Jan Kerckhofs. #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>1189</v>
+      </c>
+      <c r="I47" t="n">
+        <v>13</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>DOWNLOAD_FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>7.364334761172618e+18</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7364334761172618528</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1714642817</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2024-05-02 02:40:17</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Hoe heb jij de coronacrisis beleefd? #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>1512</v>
+      </c>
+      <c r="I48" t="n">
+        <v>20</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Ik vond het heel verregaand in ons in ons land in Onze samenleving Een avondklok instellen bijvoorbeeld alleen Wie had dat ooit kunnen denken bijna verplicht gevaccineerd worden en als je daar kritische vragen over stelde en dan word je ook ineens een anti vaxxer dus het was het was het was eigenlijk een beetje een Kampen verdeeld allemaal Ik vond het ook een beetje een een opbod bij momenten van wat ik doe nu dit dus Oh dan moet moet iemand anders nog verder gaan de de samenvatting voor mij is wel van de Kijk in Brussel heeft mijn heel veel beslissingen genomen maar de lokale bestuur de 600 steden en gemeenten in België eh moesten het wel allemaal bolwerken we hebben daar heel duidelijk gecommuniceerd Ik heb iedere zaterdag toen een eh een boodschap opgenomen maar de Edegem naartoe dat er die week weer zou veranderen Ik moet eerlijk zeggen ik ben heel blij dat er allemaal achter de rug is</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>7.36359344594171e+18</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7363593445941710112</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1714470213</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2024-04-30 02:43:33</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Samen veilig METsU #1: Cas Goossens van Grand Café De Rooden Hoed In aanloop naar de verkiezingen in juni 2024 ga ik elke week het gesprek aan met mensen die een verhaal te vertellen hebben en hoe ik daar vanuit de politiek tegenover sta. #kies24 #verkiezingen #politiek #antwerpen #edegem</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>17201</v>
+      </c>
+      <c r="I49" t="n">
+        <v>190</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Ze waren hier buiten aan het protesteren omdat er konijnen op jullie kaarten ik weet niet januari gecontacteerd dat dat van de kaart moest tot stalken to zeg ja ik kan niet van mijn kaarten want dat kan ik alles voor mekaar ding en dan moet ik gewoon vegetarisch restaurant gaan open doen</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>7.363277629413281e+18</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7363277629413281057</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1714396681</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2024-04-29 06:18:01</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>In Edegem deed je een moeilijke efficiëntie oefening. Hoe kijk je daar op terug?  #kies24 #nieuws #verkiezingen #politiek #edegem #antwerpen</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>1157</v>
+      </c>
+      <c r="I50" t="n">
+        <v>11</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Industrieweg 2019 Dat moest nog komen Dat wist we toen nog niet voor mij persoonlijke een heel moeilijk jaar was professioneel je zien omdat wij ja we moeten organiseren en in een lokaal bestuur in de gemeente is dat defecto al niet zo heel evident hè bij ons dat een impact op 52% van ons personeel wat gigantisch is zoals geen naakte ontslagen dus ook iedereen wil kunnen overdragen naar eh naar andere werkgevers ook met behoud van widde enzovoorts niemand is er op achteruit gaan maar wij moesten dat doen omdat wij echt waar ja de de Stroop rond onze nek voelen we hebben die beslissing genomen en momenteel begint dat ook echt wel te renderen dus we hebben eigenlijk 1,6 mln uit exploitatiekosten kunnen halen en die rechtstreeks pompen in de investeringen we hebben dat ook gedaan hè Er zijn nog nooit zoveel nieuwe voetpad Waar ligt dat we zijn bezig met de met de perkjes en zo voorts Mark moet er ook eerlijk bij zeggen Wij hebben wel 1 jaar 2 jaar echt moeten zoeken naar de juiste externe Partners dus het was noodzakelijk was het leuk eh neen want ik denk dat als als Burgemeester was politiek is de koers had het veel gemakkelijker is om zomaar verder te doen eh maar wij hebben wel twee keer de aanvullende personenbelasting kunnen doen Dalen hè dus we hebben dat echt wel voor de Edegem naar gedaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>7.361760492324392e+18</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7361760492324392224</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1714043440</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2024-04-25 04:10:40</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>#politics #fyp #tiktokvlaanderen</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>1274</v>
+      </c>
+      <c r="I51" t="n">
+        <v>38</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>DOWNLOAD_FAILED</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>7.342833628432322e+18</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7342833628432321824</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1709636725</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2024-03-05 03:05:25</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Al die politici op Tiktok en op straat: de campagne komt eraan. Maar de beste campagne? Dat is nog steeds héél je mandaat door enorm hard werken.  #politiek #tiktokvlaanderen #tafelvangert</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>1644</v>
+      </c>
+      <c r="I52" t="n">
+        <v>32</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>laten jullie je leiden door politieke reclame ja of nee ik denk wel dat hij al belangrijk is om eh zowel online als offline eh campagne te voeren en en als mensen je niet kennen kunnen ze niet u stemmen eh dus ik denk dat je dat je een beetje alleen moet gaan maar ik vind het een hele goede vraag ik had vandaag een Stedelijk Lyceum op visite perspectief uit Antwerpen in de kamer en het ging daaronder andere over hè mensen die voor de eerste keer mogen gaan stemmen maar dat is een nieuwe generatie Dat is een soort tiktok generatie moet allemaal heel snel gaan heel flashy en ik ben ik ben ben bijzonder blij eh dat dat wij hier nog nee zeggen om dat toch best wel mensen en dat je je verdiept en wat betekent die partij op wie dat je dan ook stem</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>7.342422178970815e+18</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7342422178970815776</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1709540898</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2024-03-04 00:28:18</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Ons OLVE Edegem klimaatschool van het jaar? Damn!</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>6622</v>
+      </c>
+      <c r="I53" t="n">
+        <v>70</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>weten jullie dat nog eens uitgeroepen tot de coolste klimaatschool van het jaar ik nodig Juliette op donderdag 7 maart tijdens de voormiddag speeltijd om 10:10 we gaan dan symbolisch 2 klimaat bomen planten en ik zou daar heel graag doen met de 3e graad van het OV College ook hier in Brussel heeft iedereen de mond vol over het behalen van de klimaatdoelstellingen en terecht ook maar in Edegem en meer nog in het OV Ja ze hebben de dat wordt aan het voegen dus donderdag 7 maart om 10:10 planten wij samen twee symbolische bomen voor het behalen van een mooie titel klimaatschool van het jaar Proficiat alvast in totaal</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>7.333879004660911e+18</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7333879004660911392</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>1707551789</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2024-02-09 23:56:29</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Kan een N-VA’er zich engageren voor het Belgisch leger? #fyp #tiktokvlaanderen #politiek</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>13699</v>
+      </c>
+      <c r="I54" t="n">
+        <v>230</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>kon niet helemaal anders je zit in het Belgisch leger gaat België verdedigen Maar je bent een NVA ga ik niet liever willen dan dat ons land uit elkaar valt met mekaar helemaal niet Ik ben vrede levens thuis naar iedereen kan eigenlijk vergelijken met mijn rol als Burgemeester er zijn ook mensen in Edegem die die niet op mij of op mijn partij gestemd hebben en ik ik wensen zij en ook het beste toen ik werk ook dat en dat gaat voor voor hun en dat is in België en anders wat niet wil zeggen eh dat ik het ben met onze Belgische politicus structuur die volledig kentucky's eh dat gaat wel ge verdedigen als het moet maar ik zal the wall verdedigen eh even zeggen dat ik die Vlaming verdediging ik ben ik ben legalist ik ben op tot op heden op mijn identiteitskaart eh Belg eh nogmaals ik herhaal wat niet wil zeggen dat ik akkoord ben met hoe dat ons land werkt of niet werkt</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>7.333556945367993e+18</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7333556945367993633</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>1707476794</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2024-02-09 03:06:34</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Gisteren bij Gert uitgelegd wat reservisten bij het leger zijn en wat wij doen. @GoPlay</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>3040</v>
+      </c>
+      <c r="I55" t="n">
+        <v>35</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>eh in 2019 heb ik aan de kms de Koninklijke Militaire school mijn hogere studies voor Veiligheid en Defensie mogen doen in het diagon heet dat de 4e cyclus en daar eigenlijk Ja dat zijn mijn ogen toch wel een beetje open gaan over eh De Burgerij versus eh Defensie en daar was een generaal bij is nu Generaal geworden die mij zo dat laatste pushy gegeven heeft van wij kunnen nu gebruiken kwam een joinus En dan begint hij nu parcours natuurlijk niet zo evident uh parcours bedoelt een soort opleiding ja ja ja kunnen we dat vergelijken met wat we zien in kamp Waes ehm de Lite versie je leert vuren je leert techniek tactiek je gaat bivakkeren die teamgeest jou nu heel scherp eh maar je wordt wel fysiek en mentaal toch wel uitgedaagd en dat durf ik wel eh durf ik wel zeggen Ik kan je nu bijvoorbeeld elk moment hier opgeroepen worden verdien of dat zou kunnen maar dat gaat niet gebeuren toch moet je bereid zijn om eventueel te gaan vechten Dat is een eed die eh die af ligt want eigenlijk is het zo dat als burger eigenlijk jouw expertise mee kunnen inzetten voor Defensie dat dat ook die kloof tussen Defensie en dat lijkt zo ver weg ook dat je die een stukje kan dichten en de waarde de normen het respecte de discipline bij defensie Ik moet heel eerlijk zeggen dat je mij ook nog wel eens dicht</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>7.330569546044165e+18</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7330569546044165408</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>1706781236</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2024-02-01 01:53:56</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Vandaag ondertekenden we het jongerenparticipatiecharter. #politiek #parlement #tiktokvlaanderen</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>7200</v>
+      </c>
+      <c r="I56" t="n">
+        <v>79</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>7.329260044573232e+18</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7329260044573232416</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>1706476341</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2024-01-28 13:12:21</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>2323</v>
+      </c>
+      <c r="I57" t="n">
+        <v>15</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>7.326293865621622e+18</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@koen.metsu.tiktok/video/7326293865621622049</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1705785722</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2024-01-20 13:22:02</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Dagje Ardennen, pijnlijk plezant.#fyp #tiktokvlaanderen</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>koen.metsu.tiktok</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>2081</v>
+      </c>
+      <c r="I58" t="n">
+        <v>22</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>NO_SPEECH_DETECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>kathleen.depoorter</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>7329940889671896352</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
+      <c r="B59" t="n">
+        <v>7.34889949532683e+18</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@kathleen.depoorter/video/7348899495326829856</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>1711049062</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2024-03-21 12:24:22</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Preventie, vroege diagnose en nieuwe therapieën zijn essentieel in de strijd tegen #kanker. Als N-VA pleiten we voor een nieuw kankerplan met een gerichte aanpak en bijzondere aandacht voor prostaatkanker en longkanker.</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>kathleen.depoorter</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>390</v>
+      </c>
+      <c r="I59" t="n">
+        <v>12</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>in ons land sterven nog veel te veel mensen aan kanker en toch hebben we geen geactualiseerd kanker plan We zetten in op preventie tegen borstkanker en dikke darmkanker maar te weinig mensen in een deel aan de screening programma's Bovendien is het zo dat we voor prostaatkanker en longkanker geen plan hebben wij als een via willen inzetten op een vroege detectie voor prostaatkanker en longkanker Ja we willen werk maken van een nieuw Nationaal kanker plan aangepast aan de noten van vandaag waren we inzetten op preventie vroege diagnose en nieuwe therapieën Zo kunnen we samen de strijd aangaan tegen kanker</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>kathleen.depoorter</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>7.340979348725304e+18</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@kathleen.depoorter/video/7340979348725304609</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>1709204963</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2024-02-29 03:09:23</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Regelmatig krijg ik vragen over #Ozempic. Als apotheker en #parlementslid ben ik me bewust van het tekort, niet alleen van Ozempic-pennen, maar ook van andere #medicatie. Om dit probleem aan te pakken, heeft de #N-VA enkele jaren geleden een wetsvoorstel ingediend. Het voorstel is ondertussen goedgekeurd maar de uitvoering ervan door Minister Vandenbroucke laat nog op zich wachten. Ik volg het alvast op voor u!</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>kathleen.depoorter</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>93</v>
+      </c>
+      <c r="I60" t="n">
+        <v>7</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Ik krijg de laatste tijd wel vaker vragen over OZ en pik de spuiten diabetes patiënten nodig hebben om een suikerziekte te behandelen en waar je ook wel van kan vermageren ik bestellen op het internet is echt geen goed idee want je hebt geen garantie van de kwaliteiten heb je enkel op voorschrift en bij de apotheek er zijn ook veel valse Oh zijn pik pennen in omloop en dat kan echt gevaarlijk zijn voor de gezondheid nu als NVA hebben wij een wet voorstel ingediend en goedgekeurd rond ontbrekende geneesmiddelen want dat is echt wel een probleem Het is goedgekeurde uitvoering daar wachten we nog op die moet gebeuren door minister van den broecke maar ik volg het voor u verderop hier in het parlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>kathleen.depoorter</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>7.338354886922391e+18</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@kathleen.depoorter/video/7338354886922390816</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>1708593935</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2024-02-22 01:25:35</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>1048 #jongeren tussen 18 en 24 jaar werden er in 2021 in gedwongen opnames geplaatst. Dat zijn er 35% meer dan in het jaar 2017. Deze stijging is het zoveelste signaal dat het niet goed gaat met het mentaal welzijn van onze jeugd. Er moet dringend meer ingezet worden op #preventie en sensibilisering, meer ambulante zorg en we hebben nood aan meer zorgverstrekkers gespecialiseerd in geestelijke #gezondheidszorg !</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>kathleen.depoorter</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>912</v>
+      </c>
+      <c r="I61" t="n">
+        <v>12</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>mentaal welzijn van de Vlaming staat onder druk en de cijfers liegen er niet om bij mijn liefste een op de 5 Vlamingen worden mentale stoornissen ontdekt en al zeker over de jongeren maken we ons zorgen in het jaar 2021 werden 1048 jonge mensen in een gedwongen opname geplaatst dat is ontzettend veel als Nvidia willen we inzetten op geestelijke gezondheidszorg en we willen dat door meer preventie te gaan voorzien sensibilisering meer zorgverstrekkers die de mensen effectief kunnen helpen we willen absoluut inzetten op meneer ambulante zorg voor onze patiënt</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>kathleen.depoorter</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>7.329940889671896e+18</v>
+      </c>
+      <c r="C62" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@kathleen.depoorter/video/7329940889671896352</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="D62" t="n">
         <v>1706634867</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>2024-01-30 09:14:27</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>Wandel je even mee? 🚶‍♂️ Want tot aan de verkiezingen zal ik regelmatig wandelvideo's delen over #dossiers die ik in het parlement volg. Vandaag bespreek ik de betrokkenheid van #UNRWA-medewerkers bij de aanslag op #Israël op 7 oktober. Tien andere landen hebben reeds de #financiering stopgezet. Het is tijd dat ons land dat ook doet.</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>kathleen.depoorter</t>
         </is>
       </c>
-      <c r="H22" t="n">
+      <c r="H62" t="n">
         <v>323</v>
       </c>
-      <c r="I22" t="n">
+      <c r="I62" t="n">
         <v>11</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>undra is het agentschap van de Verenigde Naties dat de humanitaire hulp en gassa uitvoert nu blijkt dat teen van haar medewerkers meegewerkt zouden hebben aan de terroristische aanval in Israël op 7 oktober ook zo één op de 10 van de medewerkers van Linkin hebben met gras ondertussen hebben meer dan 10 landen samenwerking met het organisatie stopgezet Wij vragen minister Guinee om een onderzoek uit te voeren en tot dan die financiering van de humanitaire hulp op te schorten je kan bijvoorbeeld via het Rode Kruis gaan werken en ervoor zorgen dat er toch middelen naar de mensen gaan die ze echt nodig hebben we hebben de minister eerder gewaarschuwd maar er is niks gebeurd Laat ons de zaken aanpakken en er voor zorgen dat ons belastinggeld komt daar waar het echt kan helpen</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>